<commit_message>
fix: synchronize report timestamps with actual last_updated.txt scraper time
</commit_message>
<xml_diff>
--- a/dashboard/public/Report_Dashboard_Latest.xlsx
+++ b/dashboard/public/Report_Dashboard_Latest.xlsx
@@ -541,14 +541,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hari/Tanggal : Kamis, 18 Juli 2026</t>
+          <t>Hari/Tanggal : 18 Juli 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 15:21 WITA</t>
+          <t>Pukul        : 06.55 WITA</t>
         </is>
       </c>
     </row>
@@ -1807,14 +1807,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hari/Tanggal : Kamis, 18 Juli 2026</t>
+          <t>Hari/Tanggal : 18 Juli 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 15:21 WITA</t>
+          <t>Pukul        : 06.55 WITA</t>
         </is>
       </c>
     </row>
@@ -8036,14 +8036,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hari/Tanggal : Kamis, 18 Juli 2026</t>
+          <t>Hari/Tanggal : 18 Juli 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 15:21 WITA</t>
+          <t>Pukul        : 06.55 WITA</t>
         </is>
       </c>
     </row>
@@ -9227,14 +9227,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hari/Tanggal : Kamis, 18 Juli 2026</t>
+          <t>Hari/Tanggal : 18 Juli 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 15:21 WITA</t>
+          <t>Pukul        : 06.55 WITA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data: 19 Juli 2026 pukul 11.58 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Report_Dashboard_Latest.xlsx
+++ b/dashboard/public/Report_Dashboard_Latest.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Monitoring Kecamatan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Leaderboard PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Leaderboard PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Leaderboard Kecamatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring Kecamatan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leaderboard PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leaderboard PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leaderboard Kecamatan" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -610,7 +610,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 11.52 WITA</t>
+          <t>Pukul        : 11.58 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1911,7 +1911,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 11.52 WITA</t>
+          <t>Pukul        : 11.58 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -8160,7 +8160,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 11.52 WITA</t>
+          <t>Pukul        : 11.58 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -9371,7 +9371,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 11.52 WITA</t>
+          <t>Pukul        : 11.58 WITA</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update data mikro SLS and sync dashboard: 10 Agustus 2026 pukul 13.03 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Report_Dashboard_Latest.xlsx
+++ b/dashboard/public/Report_Dashboard_Latest.xlsx
@@ -80,11 +80,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C6500"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C0006"/>
+      <color rgb="009C6500"/>
     </font>
     <font>
       <b val="1"/>
@@ -167,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -181,14 +181,12 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="9" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="10" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="10" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="11" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="12" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -618,32 +616,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 08.13 WITA</t>
+          <t>Pukul        : 13.03 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Target Hari Ini (H-56):</t>
+          <t>Target Hari Ini (H-57):</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>93.52%</t>
+          <t>95.19%</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Hijau &gt;= 93.52%</t>
+          <t>Hijau &gt;= 95.19%</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Kuning 46.76% - 93.52%</t>
+          <t>Kuning 47.59% - 95.19%</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Merah &lt; 46.76%</t>
+          <t>Merah &lt; 47.59%</t>
         </is>
       </c>
     </row>
@@ -807,7 +805,7 @@
         <v/>
       </c>
       <c r="R7" s="9" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="S7" s="13">
         <f>R7/B7</f>
@@ -871,12 +869,12 @@
       <c r="P8" s="10" t="n">
         <v>1358</v>
       </c>
-      <c r="Q8" s="13">
+      <c r="Q8" s="14">
         <f>P8/B8</f>
         <v/>
       </c>
       <c r="R8" s="9" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="S8" s="13">
         <f>R8/B8</f>
@@ -884,7 +882,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Tamako</t>
         </is>
@@ -944,16 +942,16 @@
         <f>P9/B9</f>
         <v/>
       </c>
-      <c r="R9" s="14" t="n">
-        <v>42</v>
-      </c>
-      <c r="S9" s="15">
+      <c r="R9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="13">
         <f>R9/B9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Tabukan Selatan</t>
         </is>
@@ -1013,16 +1011,16 @@
         <f>P10/B10</f>
         <v/>
       </c>
-      <c r="R10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" s="15">
+      <c r="R10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="13">
         <f>R10/B10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Tabukan Selatan Tengah</t>
         </is>
@@ -1078,20 +1076,20 @@
       <c r="P11" s="10" t="n">
         <v>1100</v>
       </c>
-      <c r="Q11" s="13">
+      <c r="Q11" s="14">
         <f>P11/B11</f>
         <v/>
       </c>
-      <c r="R11" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="S11" s="15">
+      <c r="R11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="13">
         <f>R11/B11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Tabukan Selatan Tenggara</t>
         </is>
@@ -1151,16 +1149,16 @@
         <f>P12/B12</f>
         <v/>
       </c>
-      <c r="R12" s="16" t="n">
-        <v>30</v>
-      </c>
-      <c r="S12" s="12">
+      <c r="R12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="13">
         <f>R12/B12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Tabukan Tengah</t>
         </is>
@@ -1216,14 +1214,14 @@
       <c r="P13" s="10" t="n">
         <v>4454</v>
       </c>
-      <c r="Q13" s="13">
+      <c r="Q13" s="14">
         <f>P13/B13</f>
         <v/>
       </c>
-      <c r="R13" s="16" t="n">
-        <v>143</v>
-      </c>
-      <c r="S13" s="12">
+      <c r="R13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="13">
         <f>R13/B13</f>
         <v/>
       </c>
@@ -1285,12 +1283,12 @@
       <c r="P14" s="10" t="n">
         <v>5922</v>
       </c>
-      <c r="Q14" s="13">
+      <c r="Q14" s="14">
         <f>P14/B14</f>
         <v/>
       </c>
       <c r="R14" s="9" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="S14" s="13">
         <f>R14/B14</f>
@@ -1298,7 +1296,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Tahuna</t>
         </is>
@@ -1354,14 +1352,14 @@
       <c r="P15" s="10" t="n">
         <v>7978</v>
       </c>
-      <c r="Q15" s="13">
+      <c r="Q15" s="14">
         <f>P15/B15</f>
         <v/>
       </c>
-      <c r="R15" s="16" t="n">
-        <v>184</v>
-      </c>
-      <c r="S15" s="12">
+      <c r="R15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="13">
         <f>R15/B15</f>
         <v/>
       </c>
@@ -1423,12 +1421,12 @@
       <c r="P16" s="10" t="n">
         <v>5090</v>
       </c>
-      <c r="Q16" s="13">
+      <c r="Q16" s="14">
         <f>P16/B16</f>
         <v/>
       </c>
       <c r="R16" s="9" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="S16" s="13">
         <f>R16/B16</f>
@@ -1436,7 +1434,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Tahuna Barat</t>
         </is>
@@ -1492,20 +1490,20 @@
       <c r="P17" s="10" t="n">
         <v>2250</v>
       </c>
-      <c r="Q17" s="13">
+      <c r="Q17" s="14">
         <f>P17/B17</f>
         <v/>
       </c>
-      <c r="R17" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="S17" s="15">
+      <c r="R17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="13">
         <f>R17/B17</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Tabukan Utara</t>
         </is>
@@ -1565,16 +1563,16 @@
         <f>P18/B18</f>
         <v/>
       </c>
-      <c r="R18" s="14" t="n">
-        <v>83</v>
-      </c>
-      <c r="S18" s="15">
+      <c r="R18" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="13">
         <f>R18/B18</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Nusa Tabukan</t>
         </is>
@@ -1634,16 +1632,16 @@
         <f>P19/B19</f>
         <v/>
       </c>
-      <c r="R19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" s="15">
+      <c r="R19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="13">
         <f>R19/B19</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Kepulauan Marore</t>
         </is>
@@ -1699,20 +1697,20 @@
       <c r="P20" s="10" t="n">
         <v>435</v>
       </c>
-      <c r="Q20" s="13">
+      <c r="Q20" s="14">
         <f>P20/B20</f>
         <v/>
       </c>
-      <c r="R20" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" s="15">
+      <c r="R20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="13">
         <f>R20/B20</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>Kendahe</t>
         </is>
@@ -1768,14 +1766,14 @@
       <c r="P21" s="10" t="n">
         <v>2758</v>
       </c>
-      <c r="Q21" s="13">
+      <c r="Q21" s="14">
         <f>P21/B21</f>
         <v/>
       </c>
-      <c r="R21" s="16" t="n">
-        <v>60</v>
-      </c>
-      <c r="S21" s="12">
+      <c r="R21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="13">
         <f>R21/B21</f>
         <v/>
       </c>
@@ -1786,67 +1784,67 @@
           <t>Kab. Kepl. Sangihe</t>
         </is>
       </c>
-      <c r="B22" s="17">
+      <c r="B22" s="15">
         <f>SUM(B7:B21)</f>
         <v/>
       </c>
-      <c r="C22" s="17">
+      <c r="C22" s="15">
         <f>SUM(C7:C21)</f>
         <v/>
       </c>
-      <c r="D22" s="17">
+      <c r="D22" s="15">
         <f>SUM(D7:D21)</f>
         <v/>
       </c>
-      <c r="E22" s="18">
+      <c r="E22" s="16">
         <f>D22/B22</f>
         <v/>
       </c>
-      <c r="F22" s="17">
+      <c r="F22" s="15">
         <f>SUM(F7:F21)</f>
         <v/>
       </c>
-      <c r="G22" s="18">
+      <c r="G22" s="16">
         <f>F22/B22</f>
         <v/>
       </c>
-      <c r="H22" s="17">
+      <c r="H22" s="15">
         <f>SUM(H7:H21)</f>
         <v/>
       </c>
-      <c r="I22" s="18">
+      <c r="I22" s="16">
         <f>H22/B22</f>
         <v/>
       </c>
-      <c r="J22" s="17">
+      <c r="J22" s="15">
         <f>SUM(J7:J21)</f>
         <v/>
       </c>
-      <c r="K22" s="18">
+      <c r="K22" s="16">
         <f>J22/B22</f>
         <v/>
       </c>
-      <c r="L22" s="17">
+      <c r="L22" s="15">
         <f>SUM(L7:L21)</f>
         <v/>
       </c>
-      <c r="M22" s="18">
+      <c r="M22" s="16">
         <f>L22/B22</f>
         <v/>
       </c>
-      <c r="N22" s="17">
+      <c r="N22" s="15">
         <f>SUM(N7:N21)</f>
         <v/>
       </c>
-      <c r="O22" s="18">
+      <c r="O22" s="16">
         <f>N22/B22</f>
         <v/>
       </c>
-      <c r="P22" s="17">
+      <c r="P22" s="15">
         <f>SUM(P7:P21)</f>
         <v/>
       </c>
-      <c r="Q22" s="13">
+      <c r="Q22" s="14">
         <f>P22/B22</f>
         <v/>
       </c>
@@ -1892,7 +1890,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>LEADERBOARD PROGRES PENDATAAN LAPANGAN SE2026 MENURUT PPL</t>
         </is>
@@ -1919,83 +1917,83 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 08.13 WITA</t>
+          <t>Pukul        : 13.03 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Target Hari Ini (H-56):</t>
+          <t>Target Hari Ini (H-57):</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>93.52%</t>
+          <t>95.19%</t>
         </is>
       </c>
     </row>
     <row r="5"/>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>NAMA</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>KECAMATAN</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>KOSEKA</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>TARGET</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="F6" s="18" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="G6" s="20" t="inlineStr">
+      <c r="G6" s="18" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>
       </c>
-      <c r="H6" s="20" t="inlineStr">
+      <c r="H6" s="18" t="inlineStr">
         <is>
           <t>SUBMIT</t>
         </is>
       </c>
-      <c r="I6" s="20" t="inlineStr">
+      <c r="I6" s="18" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="J6" s="20" t="inlineStr">
+      <c r="J6" s="18" t="inlineStr">
         <is>
           <t>APPROVED</t>
         </is>
       </c>
-      <c r="K6" s="20" t="inlineStr">
+      <c r="K6" s="18" t="inlineStr">
         <is>
           <t>PROGRES</t>
         </is>
       </c>
-      <c r="L6" s="20" t="inlineStr">
+      <c r="L6" s="18" t="inlineStr">
         <is>
           <t>REALISASI</t>
         </is>
       </c>
-      <c r="M6" s="20" t="inlineStr">
+      <c r="M6" s="18" t="inlineStr">
         <is>
           <t>REALISASI (%)</t>
         </is>
@@ -4817,7 +4815,7 @@
       <c r="L66" s="10" t="n">
         <v>518</v>
       </c>
-      <c r="M66" s="12" t="n">
+      <c r="M66" s="14" t="n">
         <v>0.9504587155963303</v>
       </c>
     </row>
@@ -4864,7 +4862,7 @@
       <c r="L67" s="10" t="n">
         <v>364</v>
       </c>
-      <c r="M67" s="12" t="n">
+      <c r="M67" s="14" t="n">
         <v>0.9503916449086163</v>
       </c>
     </row>
@@ -4911,7 +4909,7 @@
       <c r="L68" s="10" t="n">
         <v>505</v>
       </c>
-      <c r="M68" s="12" t="n">
+      <c r="M68" s="14" t="n">
         <v>0.9474671669793621</v>
       </c>
     </row>
@@ -4958,7 +4956,7 @@
       <c r="L69" s="10" t="n">
         <v>554</v>
       </c>
-      <c r="M69" s="12" t="n">
+      <c r="M69" s="14" t="n">
         <v>0.9437819420783646</v>
       </c>
     </row>
@@ -5005,7 +5003,7 @@
       <c r="L70" s="10" t="n">
         <v>398</v>
       </c>
-      <c r="M70" s="12" t="n">
+      <c r="M70" s="14" t="n">
         <v>0.943127962085308</v>
       </c>
     </row>
@@ -5052,7 +5050,7 @@
       <c r="L71" s="10" t="n">
         <v>486</v>
       </c>
-      <c r="M71" s="12" t="n">
+      <c r="M71" s="14" t="n">
         <v>0.9418604651162791</v>
       </c>
     </row>
@@ -5099,7 +5097,7 @@
       <c r="L72" s="10" t="n">
         <v>427</v>
       </c>
-      <c r="M72" s="12" t="n">
+      <c r="M72" s="14" t="n">
         <v>0.9384615384615383</v>
       </c>
     </row>
@@ -5146,7 +5144,7 @@
       <c r="L73" s="10" t="n">
         <v>447</v>
       </c>
-      <c r="M73" s="12" t="n">
+      <c r="M73" s="14" t="n">
         <v>0.9371069182389937</v>
       </c>
     </row>
@@ -5193,7 +5191,7 @@
       <c r="L74" s="10" t="n">
         <v>478</v>
       </c>
-      <c r="M74" s="13" t="n">
+      <c r="M74" s="14" t="n">
         <v>0.9299610894941633</v>
       </c>
     </row>
@@ -5240,7 +5238,7 @@
       <c r="L75" s="10" t="n">
         <v>409</v>
       </c>
-      <c r="M75" s="13" t="n">
+      <c r="M75" s="14" t="n">
         <v>0.9295454545454546</v>
       </c>
     </row>
@@ -5287,7 +5285,7 @@
       <c r="L76" s="10" t="n">
         <v>377</v>
       </c>
-      <c r="M76" s="13" t="n">
+      <c r="M76" s="14" t="n">
         <v>0.9285714285714286</v>
       </c>
     </row>
@@ -5334,7 +5332,7 @@
       <c r="L77" s="10" t="n">
         <v>479</v>
       </c>
-      <c r="M77" s="13" t="n">
+      <c r="M77" s="14" t="n">
         <v>0.9282945736434108</v>
       </c>
     </row>
@@ -5381,7 +5379,7 @@
       <c r="L78" s="10" t="n">
         <v>592</v>
       </c>
-      <c r="M78" s="13" t="n">
+      <c r="M78" s="14" t="n">
         <v>0.9278996865203761</v>
       </c>
     </row>
@@ -5428,7 +5426,7 @@
       <c r="L79" s="10" t="n">
         <v>507</v>
       </c>
-      <c r="M79" s="13" t="n">
+      <c r="M79" s="14" t="n">
         <v>0.9218181818181819</v>
       </c>
     </row>
@@ -5475,7 +5473,7 @@
       <c r="L80" s="10" t="n">
         <v>518</v>
       </c>
-      <c r="M80" s="13" t="n">
+      <c r="M80" s="14" t="n">
         <v>0.9217081850533808</v>
       </c>
     </row>
@@ -5522,7 +5520,7 @@
       <c r="L81" s="10" t="n">
         <v>452</v>
       </c>
-      <c r="M81" s="13" t="n">
+      <c r="M81" s="14" t="n">
         <v>0.9186991869918699</v>
       </c>
     </row>
@@ -5569,7 +5567,7 @@
       <c r="L82" s="10" t="n">
         <v>438</v>
       </c>
-      <c r="M82" s="13" t="n">
+      <c r="M82" s="14" t="n">
         <v>0.9182389937106918</v>
       </c>
     </row>
@@ -5616,7 +5614,7 @@
       <c r="L83" s="10" t="n">
         <v>499</v>
       </c>
-      <c r="M83" s="13" t="n">
+      <c r="M83" s="14" t="n">
         <v>0.9172794117647058</v>
       </c>
     </row>
@@ -5663,7 +5661,7 @@
       <c r="L84" s="10" t="n">
         <v>433</v>
       </c>
-      <c r="M84" s="13" t="n">
+      <c r="M84" s="14" t="n">
         <v>0.915433403805497</v>
       </c>
     </row>
@@ -5710,7 +5708,7 @@
       <c r="L85" s="10" t="n">
         <v>435</v>
       </c>
-      <c r="M85" s="13" t="n">
+      <c r="M85" s="14" t="n">
         <v>0.9138655462184873</v>
       </c>
     </row>
@@ -5757,7 +5755,7 @@
       <c r="L86" s="10" t="n">
         <v>488</v>
       </c>
-      <c r="M86" s="13" t="n">
+      <c r="M86" s="14" t="n">
         <v>0.9138576779026217</v>
       </c>
     </row>
@@ -5804,7 +5802,7 @@
       <c r="L87" s="10" t="n">
         <v>483</v>
       </c>
-      <c r="M87" s="13" t="n">
+      <c r="M87" s="14" t="n">
         <v>0.9113207547169812</v>
       </c>
     </row>
@@ -5851,7 +5849,7 @@
       <c r="L88" s="10" t="n">
         <v>513</v>
       </c>
-      <c r="M88" s="13" t="n">
+      <c r="M88" s="14" t="n">
         <v>0.9063604240282686</v>
       </c>
     </row>
@@ -5898,7 +5896,7 @@
       <c r="L89" s="10" t="n">
         <v>443</v>
       </c>
-      <c r="M89" s="13" t="n">
+      <c r="M89" s="14" t="n">
         <v>0.9059304703476482</v>
       </c>
     </row>
@@ -5945,7 +5943,7 @@
       <c r="L90" s="10" t="n">
         <v>343</v>
       </c>
-      <c r="M90" s="13" t="n">
+      <c r="M90" s="14" t="n">
         <v>0.9026315789473685</v>
       </c>
     </row>
@@ -5992,7 +5990,7 @@
       <c r="L91" s="10" t="n">
         <v>422</v>
       </c>
-      <c r="M91" s="13" t="n">
+      <c r="M91" s="14" t="n">
         <v>0.9017094017094017</v>
       </c>
     </row>
@@ -6039,7 +6037,7 @@
       <c r="L92" s="10" t="n">
         <v>459</v>
       </c>
-      <c r="M92" s="13" t="n">
+      <c r="M92" s="14" t="n">
         <v>0.8982387475538161</v>
       </c>
     </row>
@@ -6086,7 +6084,7 @@
       <c r="L93" s="10" t="n">
         <v>362</v>
       </c>
-      <c r="M93" s="13" t="n">
+      <c r="M93" s="14" t="n">
         <v>0.8938271604938273</v>
       </c>
     </row>
@@ -6133,7 +6131,7 @@
       <c r="L94" s="10" t="n">
         <v>589</v>
       </c>
-      <c r="M94" s="13" t="n">
+      <c r="M94" s="14" t="n">
         <v>0.8897280966767371</v>
       </c>
     </row>
@@ -6180,7 +6178,7 @@
       <c r="L95" s="10" t="n">
         <v>408</v>
       </c>
-      <c r="M95" s="13" t="n">
+      <c r="M95" s="14" t="n">
         <v>0.8888888888888888</v>
       </c>
     </row>
@@ -6227,7 +6225,7 @@
       <c r="L96" s="10" t="n">
         <v>485</v>
       </c>
-      <c r="M96" s="13" t="n">
+      <c r="M96" s="14" t="n">
         <v>0.886654478976234</v>
       </c>
     </row>
@@ -6274,7 +6272,7 @@
       <c r="L97" s="10" t="n">
         <v>289</v>
       </c>
-      <c r="M97" s="13" t="n">
+      <c r="M97" s="14" t="n">
         <v>0.8865030674846625</v>
       </c>
     </row>
@@ -6321,7 +6319,7 @@
       <c r="L98" s="10" t="n">
         <v>468</v>
       </c>
-      <c r="M98" s="13" t="n">
+      <c r="M98" s="14" t="n">
         <v>0.8863636363636364</v>
       </c>
     </row>
@@ -6368,7 +6366,7 @@
       <c r="L99" s="10" t="n">
         <v>440</v>
       </c>
-      <c r="M99" s="13" t="n">
+      <c r="M99" s="14" t="n">
         <v>0.8853118712273642</v>
       </c>
     </row>
@@ -6415,7 +6413,7 @@
       <c r="L100" s="10" t="n">
         <v>392</v>
       </c>
-      <c r="M100" s="13" t="n">
+      <c r="M100" s="14" t="n">
         <v>0.8848758465011286</v>
       </c>
     </row>
@@ -6462,7 +6460,7 @@
       <c r="L101" s="10" t="n">
         <v>405</v>
       </c>
-      <c r="M101" s="13" t="n">
+      <c r="M101" s="14" t="n">
         <v>0.8842794759825326</v>
       </c>
     </row>
@@ -6509,7 +6507,7 @@
       <c r="L102" s="10" t="n">
         <v>376</v>
       </c>
-      <c r="M102" s="13" t="n">
+      <c r="M102" s="14" t="n">
         <v>0.8826291079812206</v>
       </c>
     </row>
@@ -6556,7 +6554,7 @@
       <c r="L103" s="10" t="n">
         <v>406</v>
       </c>
-      <c r="M103" s="13" t="n">
+      <c r="M103" s="14" t="n">
         <v>0.8768898488120951</v>
       </c>
     </row>
@@ -6603,7 +6601,7 @@
       <c r="L104" s="10" t="n">
         <v>418</v>
       </c>
-      <c r="M104" s="13" t="n">
+      <c r="M104" s="14" t="n">
         <v>0.872651356993737</v>
       </c>
     </row>
@@ -6650,7 +6648,7 @@
       <c r="L105" s="10" t="n">
         <v>390</v>
       </c>
-      <c r="M105" s="13" t="n">
+      <c r="M105" s="14" t="n">
         <v>0.8724832214765101</v>
       </c>
     </row>
@@ -6697,7 +6695,7 @@
       <c r="L106" s="10" t="n">
         <v>366</v>
       </c>
-      <c r="M106" s="13" t="n">
+      <c r="M106" s="14" t="n">
         <v>0.8714285714285714</v>
       </c>
     </row>
@@ -6744,7 +6742,7 @@
       <c r="L107" s="10" t="n">
         <v>366</v>
       </c>
-      <c r="M107" s="13" t="n">
+      <c r="M107" s="14" t="n">
         <v>0.8714285714285714</v>
       </c>
     </row>
@@ -6791,7 +6789,7 @@
       <c r="L108" s="10" t="n">
         <v>382</v>
       </c>
-      <c r="M108" s="13" t="n">
+      <c r="M108" s="14" t="n">
         <v>0.8681818181818182</v>
       </c>
     </row>
@@ -6838,7 +6836,7 @@
       <c r="L109" s="10" t="n">
         <v>497</v>
       </c>
-      <c r="M109" s="13" t="n">
+      <c r="M109" s="14" t="n">
         <v>0.8658536585365852</v>
       </c>
     </row>
@@ -6885,7 +6883,7 @@
       <c r="L110" s="10" t="n">
         <v>323</v>
       </c>
-      <c r="M110" s="13" t="n">
+      <c r="M110" s="14" t="n">
         <v>0.8636363636363636</v>
       </c>
     </row>
@@ -6932,7 +6930,7 @@
       <c r="L111" s="10" t="n">
         <v>373</v>
       </c>
-      <c r="M111" s="13" t="n">
+      <c r="M111" s="14" t="n">
         <v>0.8555045871559633</v>
       </c>
     </row>
@@ -6979,7 +6977,7 @@
       <c r="L112" s="10" t="n">
         <v>459</v>
       </c>
-      <c r="M112" s="13" t="n">
+      <c r="M112" s="14" t="n">
         <v>0.8547486033519553</v>
       </c>
     </row>
@@ -7026,7 +7024,7 @@
       <c r="L113" s="10" t="n">
         <v>444</v>
       </c>
-      <c r="M113" s="13" t="n">
+      <c r="M113" s="14" t="n">
         <v>0.8538461538461539</v>
       </c>
     </row>
@@ -7073,7 +7071,7 @@
       <c r="L114" s="10" t="n">
         <v>463</v>
       </c>
-      <c r="M114" s="13" t="n">
+      <c r="M114" s="14" t="n">
         <v>0.852670349907919</v>
       </c>
     </row>
@@ -7120,7 +7118,7 @@
       <c r="L115" s="10" t="n">
         <v>448</v>
       </c>
-      <c r="M115" s="13" t="n">
+      <c r="M115" s="14" t="n">
         <v>0.8517110266159694</v>
       </c>
     </row>
@@ -7167,7 +7165,7 @@
       <c r="L116" s="10" t="n">
         <v>378</v>
       </c>
-      <c r="M116" s="13" t="n">
+      <c r="M116" s="14" t="n">
         <v>0.8513513513513513</v>
       </c>
     </row>
@@ -7214,7 +7212,7 @@
       <c r="L117" s="10" t="n">
         <v>418</v>
       </c>
-      <c r="M117" s="13" t="n">
+      <c r="M117" s="14" t="n">
         <v>0.8513238289205702</v>
       </c>
     </row>
@@ -7261,7 +7259,7 @@
       <c r="L118" s="10" t="n">
         <v>412</v>
       </c>
-      <c r="M118" s="13" t="n">
+      <c r="M118" s="14" t="n">
         <v>0.8512396694214877</v>
       </c>
     </row>
@@ -7308,7 +7306,7 @@
       <c r="L119" s="10" t="n">
         <v>441</v>
       </c>
-      <c r="M119" s="13" t="n">
+      <c r="M119" s="14" t="n">
         <v>0.8497109826589595</v>
       </c>
     </row>
@@ -7355,7 +7353,7 @@
       <c r="L120" s="10" t="n">
         <v>403</v>
       </c>
-      <c r="M120" s="13" t="n">
+      <c r="M120" s="14" t="n">
         <v>0.8448637316561844</v>
       </c>
     </row>
@@ -7402,7 +7400,7 @@
       <c r="L121" s="10" t="n">
         <v>399</v>
       </c>
-      <c r="M121" s="13" t="n">
+      <c r="M121" s="14" t="n">
         <v>0.8382352941176471</v>
       </c>
     </row>
@@ -7449,7 +7447,7 @@
       <c r="L122" s="10" t="n">
         <v>430</v>
       </c>
-      <c r="M122" s="13" t="n">
+      <c r="M122" s="14" t="n">
         <v>0.8382066276803118</v>
       </c>
     </row>
@@ -7496,7 +7494,7 @@
       <c r="L123" s="10" t="n">
         <v>403</v>
       </c>
-      <c r="M123" s="13" t="n">
+      <c r="M123" s="14" t="n">
         <v>0.8378378378378379</v>
       </c>
     </row>
@@ -7543,7 +7541,7 @@
       <c r="L124" s="10" t="n">
         <v>303</v>
       </c>
-      <c r="M124" s="13" t="n">
+      <c r="M124" s="14" t="n">
         <v>0.8324175824175825</v>
       </c>
     </row>
@@ -7590,7 +7588,7 @@
       <c r="L125" s="10" t="n">
         <v>387</v>
       </c>
-      <c r="M125" s="13" t="n">
+      <c r="M125" s="14" t="n">
         <v>0.8322580645161292</v>
       </c>
     </row>
@@ -7637,7 +7635,7 @@
       <c r="L126" s="10" t="n">
         <v>377</v>
       </c>
-      <c r="M126" s="13" t="n">
+      <c r="M126" s="14" t="n">
         <v>0.8303964757709251</v>
       </c>
     </row>
@@ -7684,7 +7682,7 @@
       <c r="L127" s="10" t="n">
         <v>449</v>
       </c>
-      <c r="M127" s="13" t="n">
+      <c r="M127" s="14" t="n">
         <v>0.8253676470588235</v>
       </c>
     </row>
@@ -7731,7 +7729,7 @@
       <c r="L128" s="10" t="n">
         <v>380</v>
       </c>
-      <c r="M128" s="13" t="n">
+      <c r="M128" s="14" t="n">
         <v>0.824295010845987</v>
       </c>
     </row>
@@ -7778,7 +7776,7 @@
       <c r="L129" s="10" t="n">
         <v>427</v>
       </c>
-      <c r="M129" s="13" t="n">
+      <c r="M129" s="14" t="n">
         <v>0.8211538461538461</v>
       </c>
     </row>
@@ -7825,7 +7823,7 @@
       <c r="L130" s="10" t="n">
         <v>389</v>
       </c>
-      <c r="M130" s="13" t="n">
+      <c r="M130" s="14" t="n">
         <v>0.820675105485232</v>
       </c>
     </row>
@@ -7872,7 +7870,7 @@
       <c r="L131" s="10" t="n">
         <v>378</v>
       </c>
-      <c r="M131" s="13" t="n">
+      <c r="M131" s="14" t="n">
         <v>0.8199566160520607</v>
       </c>
     </row>
@@ -7919,7 +7917,7 @@
       <c r="L132" s="10" t="n">
         <v>614</v>
       </c>
-      <c r="M132" s="13" t="n">
+      <c r="M132" s="14" t="n">
         <v>0.8057742782152231</v>
       </c>
     </row>
@@ -7966,7 +7964,7 @@
       <c r="L133" s="10" t="n">
         <v>484</v>
       </c>
-      <c r="M133" s="13" t="n">
+      <c r="M133" s="14" t="n">
         <v>0.8039867109634552</v>
       </c>
     </row>
@@ -8013,7 +8011,7 @@
       <c r="L134" s="10" t="n">
         <v>332</v>
       </c>
-      <c r="M134" s="13" t="n">
+      <c r="M134" s="14" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -8060,7 +8058,7 @@
       <c r="L135" s="10" t="n">
         <v>254</v>
       </c>
-      <c r="M135" s="13" t="n">
+      <c r="M135" s="14" t="n">
         <v>0.7492625368731564</v>
       </c>
     </row>
@@ -8107,7 +8105,7 @@
       <c r="L136" s="10" t="n">
         <v>435</v>
       </c>
-      <c r="M136" s="13" t="n">
+      <c r="M136" s="14" t="n">
         <v>0.6839622641509435</v>
       </c>
     </row>
@@ -8141,7 +8139,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>LEADERBOARD PROGRES PENDATAAN LAPANGAN SE2026 MENURUT PML</t>
         </is>
@@ -8168,83 +8166,83 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 08.13 WITA</t>
+          <t>Pukul        : 13.03 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Target Hari Ini (H-56):</t>
+          <t>Target Hari Ini (H-57):</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>93.52%</t>
+          <t>95.19%</t>
         </is>
       </c>
     </row>
     <row r="5"/>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>NAMA</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>KECAMATAN</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>KOSEKA</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>TARGET</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="F6" s="18" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="G6" s="20" t="inlineStr">
+      <c r="G6" s="18" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>
       </c>
-      <c r="H6" s="20" t="inlineStr">
+      <c r="H6" s="18" t="inlineStr">
         <is>
           <t>SUBMIT</t>
         </is>
       </c>
-      <c r="I6" s="20" t="inlineStr">
+      <c r="I6" s="18" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="J6" s="20" t="inlineStr">
+      <c r="J6" s="18" t="inlineStr">
         <is>
           <t>APPROVED</t>
         </is>
       </c>
-      <c r="K6" s="20" t="inlineStr">
+      <c r="K6" s="18" t="inlineStr">
         <is>
           <t>REVOKE</t>
         </is>
       </c>
-      <c r="L6" s="20" t="inlineStr">
+      <c r="L6" s="18" t="inlineStr">
         <is>
           <t>REALISASI</t>
         </is>
       </c>
-      <c r="M6" s="20" t="inlineStr">
+      <c r="M6" s="18" t="inlineStr">
         <is>
           <t>REALISASI (%)</t>
         </is>
@@ -8528,7 +8526,7 @@
       <c r="L12" s="10" t="n">
         <v>2189</v>
       </c>
-      <c r="M12" s="13" t="n">
+      <c r="M12" s="14" t="n">
         <v>0.9346712211784799</v>
       </c>
     </row>
@@ -8575,7 +8573,7 @@
       <c r="L13" s="10" t="n">
         <v>2938</v>
       </c>
-      <c r="M13" s="13" t="n">
+      <c r="M13" s="14" t="n">
         <v>0.9300411522633745</v>
       </c>
     </row>
@@ -8622,7 +8620,7 @@
       <c r="L14" s="10" t="n">
         <v>2972</v>
       </c>
-      <c r="M14" s="13" t="n">
+      <c r="M14" s="14" t="n">
         <v>0.9281698938163647</v>
       </c>
     </row>
@@ -8669,7 +8667,7 @@
       <c r="L15" s="10" t="n">
         <v>2844</v>
       </c>
-      <c r="M15" s="13" t="n">
+      <c r="M15" s="14" t="n">
         <v>0.9239766081871345</v>
       </c>
     </row>
@@ -8716,7 +8714,7 @@
       <c r="L16" s="10" t="n">
         <v>2758</v>
       </c>
-      <c r="M16" s="13" t="n">
+      <c r="M16" s="14" t="n">
         <v>0.9159747592162071</v>
       </c>
     </row>
@@ -8763,7 +8761,7 @@
       <c r="L17" s="10" t="n">
         <v>2789</v>
       </c>
-      <c r="M17" s="13" t="n">
+      <c r="M17" s="14" t="n">
         <v>0.9153265507056121</v>
       </c>
     </row>
@@ -8810,7 +8808,7 @@
       <c r="L18" s="10" t="n">
         <v>2600</v>
       </c>
-      <c r="M18" s="13" t="n">
+      <c r="M18" s="14" t="n">
         <v>0.9122807017543859</v>
       </c>
     </row>
@@ -8857,7 +8855,7 @@
       <c r="L19" s="10" t="n">
         <v>2872</v>
       </c>
-      <c r="M19" s="13" t="n">
+      <c r="M19" s="14" t="n">
         <v>0.9094363521215959</v>
       </c>
     </row>
@@ -8904,7 +8902,7 @@
       <c r="L20" s="10" t="n">
         <v>2464</v>
       </c>
-      <c r="M20" s="13" t="n">
+      <c r="M20" s="14" t="n">
         <v>0.9072164948453608</v>
       </c>
     </row>
@@ -8951,7 +8949,7 @@
       <c r="L21" s="10" t="n">
         <v>1344</v>
       </c>
-      <c r="M21" s="13" t="n">
+      <c r="M21" s="14" t="n">
         <v>0.8883013879709187</v>
       </c>
     </row>
@@ -8998,7 +8996,7 @@
       <c r="L22" s="10" t="n">
         <v>2750</v>
       </c>
-      <c r="M22" s="13" t="n">
+      <c r="M22" s="14" t="n">
         <v>0.8882428940568475</v>
       </c>
     </row>
@@ -9045,7 +9043,7 @@
       <c r="L23" s="10" t="n">
         <v>2259</v>
       </c>
-      <c r="M23" s="13" t="n">
+      <c r="M23" s="14" t="n">
         <v>0.8718641451177152</v>
       </c>
     </row>
@@ -9092,7 +9090,7 @@
       <c r="L24" s="10" t="n">
         <v>2326</v>
       </c>
-      <c r="M24" s="13" t="n">
+      <c r="M24" s="14" t="n">
         <v>0.8535779816513761</v>
       </c>
     </row>
@@ -9139,7 +9137,7 @@
       <c r="L25" s="10" t="n">
         <v>2104</v>
       </c>
-      <c r="M25" s="13" t="n">
+      <c r="M25" s="14" t="n">
         <v>0.8466800804828973</v>
       </c>
     </row>
@@ -9186,7 +9184,7 @@
       <c r="L26" s="10" t="n">
         <v>2432</v>
       </c>
-      <c r="M26" s="13" t="n">
+      <c r="M26" s="14" t="n">
         <v>0.8360261258164318</v>
       </c>
     </row>
@@ -9233,7 +9231,7 @@
       <c r="L27" s="10" t="n">
         <v>2498</v>
       </c>
-      <c r="M27" s="13" t="n">
+      <c r="M27" s="14" t="n">
         <v>0.8174083769633508</v>
       </c>
     </row>
@@ -9280,7 +9278,7 @@
       <c r="L28" s="10" t="n">
         <v>1570</v>
       </c>
-      <c r="M28" s="13" t="n">
+      <c r="M28" s="14" t="n">
         <v>0.7211759301791456</v>
       </c>
     </row>
@@ -9327,7 +9325,7 @@
       <c r="L29" s="10" t="n">
         <v>1675</v>
       </c>
-      <c r="M29" s="13" t="n">
+      <c r="M29" s="14" t="n">
         <v>0.6907216494845361</v>
       </c>
     </row>
@@ -9352,7 +9350,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>LEADERBOARD PROGRES PENDATAAN LAPANGAN SE2026 MENURUT KECAMATAN</t>
         </is>
@@ -9379,38 +9377,38 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 08.13 WITA</t>
+          <t>Pukul        : 13.03 WITA</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Target Hari Ini (H-56):</t>
+          <t>Target Hari Ini (H-57):</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>93.52%</t>
+          <t>95.19%</t>
         </is>
       </c>
     </row>
     <row r="5"/>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>KECAMATAN</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>REALISASI (%)</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>RANK CHANGE</t>
         </is>
@@ -9428,7 +9426,7 @@
       <c r="C7" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="21" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9446,7 +9444,7 @@
       <c r="C8" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="21" t="inlineStr">
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9464,7 +9462,7 @@
       <c r="C9" s="12" t="n">
         <v>0.9943870678042209</v>
       </c>
-      <c r="D9" s="21" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9482,7 +9480,7 @@
       <c r="C10" s="12" t="n">
         <v>0.9835371136998171</v>
       </c>
-      <c r="D10" s="21" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9500,7 +9498,7 @@
       <c r="C11" s="12" t="n">
         <v>0.9819091042800412</v>
       </c>
-      <c r="D11" s="21" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9518,7 +9516,7 @@
       <c r="C12" s="12" t="n">
         <v>0.9638128861429833</v>
       </c>
-      <c r="D12" s="21" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9533,12 +9531,12 @@
           <t>Kendahe</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="14" t="n">
         <v>0.9159747592162071</v>
       </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>+2</t>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -9551,10 +9549,10 @@
           <t>Tabukan Selatan Tengah</t>
         </is>
       </c>
-      <c r="C14" s="13" t="n">
+      <c r="C14" s="14" t="n">
         <v>0.9098428453267163</v>
       </c>
-      <c r="D14" s="21" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9569,12 +9567,12 @@
           <t>Tahuna Barat</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C15" s="14" t="n">
         <v>0.9054325955734407</v>
       </c>
-      <c r="D15" s="14" t="inlineStr">
-        <is>
-          <t>-2</t>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -9587,10 +9585,10 @@
           <t>Tahuna Timur</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C16" s="14" t="n">
         <v>0.9028024122029088</v>
       </c>
-      <c r="D16" s="21" t="inlineStr">
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9605,10 +9603,10 @@
           <t>Tatoareng</t>
         </is>
       </c>
-      <c r="C17" s="13" t="n">
+      <c r="C17" s="14" t="n">
         <v>0.8975545274289491</v>
       </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9623,10 +9621,10 @@
           <t>Tahuna</t>
         </is>
       </c>
-      <c r="C18" s="13" t="n">
+      <c r="C18" s="14" t="n">
         <v>0.8862475005554322</v>
       </c>
-      <c r="D18" s="21" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9641,10 +9639,10 @@
           <t>Manganitu</t>
         </is>
       </c>
-      <c r="C19" s="13" t="n">
+      <c r="C19" s="14" t="n">
         <v>0.8765541740674956</v>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9659,10 +9657,10 @@
           <t>Tabukan Tengah</t>
         </is>
       </c>
-      <c r="C20" s="13" t="n">
+      <c r="C20" s="14" t="n">
         <v>0.8537473643856621</v>
       </c>
-      <c r="D20" s="21" t="inlineStr">
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9677,10 +9675,10 @@
           <t>Kepulauan Marore</t>
         </is>
       </c>
-      <c r="C21" s="13" t="n">
+      <c r="C21" s="14" t="n">
         <v>0.6839622641509435</v>
       </c>
-      <c r="D21" s="21" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>0</t>
         </is>

</xml_diff>